<commit_message>
Selected 48 de novo UDP tubes (verified), export script, selection logic doc
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ao75Yp9yo6KZf9ARd9UmQz
</commit_message>
<xml_diff>
--- a/docs/primer_design/udp_denovo_selected_48.xlsx
+++ b/docs/primer_design/udp_denovo_selected_48.xlsx
@@ -69,12 +69,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -524,7 +524,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>48 组独立验证：最小编辑距离=4；最小反向互补距离=3；每周期全部达标=True；GC范围=(4, 6)；同聚物个数=0；序列数=96；分级 A 28 / B 20 / C 0</t>
+          <t>48 组独立验证：最小编辑距离=4；最小反向互补距离=4；每周期全部达标=True；GC范围=(4, 6)；同聚物个数=0；序列数=96；分级 A 28 / B 20 / C 0</t>
         </is>
       </c>
     </row>
@@ -749,27 +749,27 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>DN009</t>
+          <t>DN022</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>DN5009</t>
+          <t>DN5022</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>DN7009</t>
+          <t>DN7022</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>AGCCTTCACC</t>
+          <t>GCCTTACGCA</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>AGGCGCCATT</t>
+          <t>GATCACGTCG</t>
         </is>
       </c>
       <c r="G2" s="4">
@@ -782,20 +782,20 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>-6.47</v>
+        <v>-6.99</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>-4.54</v>
+        <v>-3.88</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>-1.59</v>
+        <v>-2.99</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>48970</v>
+        <v>43702</v>
       </c>
       <c r="N2" s="4" t="inlineStr"/>
       <c r="O2" s="4" t="inlineStr"/>
@@ -886,27 +886,27 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>DN022</t>
+          <t>DN023</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>DN5022</t>
+          <t>DN5023</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>DN7022</t>
+          <t>DN7023</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>GCCTTACGCA</t>
+          <t>AGTTCAGTGA</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>GATCACGTCG</t>
+          <t>TGTGTCCAAT</t>
         </is>
       </c>
       <c r="G3" s="4">
@@ -917,22 +917,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F3,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>-6.99</v>
+        <v>-6.26</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>-3.88</v>
+        <v>-3.83</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>-2.99</v>
+        <v>-1.59</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>43702</v>
+        <v>52064</v>
       </c>
       <c r="N3" s="4" t="inlineStr"/>
       <c r="O3" s="4" t="inlineStr"/>
@@ -1023,27 +1023,27 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>DN023</t>
+          <t>DN025</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>DN5023</t>
+          <t>DN5025</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>DN7023</t>
+          <t>DN7025</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>AGTTCAGTGA</t>
+          <t>CGTAGAGTCG</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>TGTGTCCAAT</t>
+          <t>GAAGGACGTC</t>
         </is>
       </c>
       <c r="G4" s="4">
@@ -1056,20 +1056,20 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>-6.26</v>
+        <v>-8.460000000000001</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>-3.83</v>
+        <v>-5.37</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>-1.59</v>
+        <v>-1.65</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>52064</v>
+        <v>268819</v>
       </c>
       <c r="N4" s="4" t="inlineStr"/>
       <c r="O4" s="4" t="inlineStr"/>
@@ -1160,27 +1160,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>DN042</t>
+          <t>DN044</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>DN5042</t>
+          <t>DN5044</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>DN7042</t>
+          <t>DN7044</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>CTGTCATGAA</t>
+          <t>AACGGACCAG</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>ATGGAGAGCC</t>
+          <t>GAATGTCTAG</t>
         </is>
       </c>
       <c r="G5" s="4">
@@ -1193,20 +1193,20 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>-6.03</v>
+        <v>-8.039999999999999</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>-3.83</v>
+        <v>-4.04</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>-1.62</v>
+        <v>-1.77</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46407</v>
+        <v>231007</v>
       </c>
       <c r="N5" s="4" t="inlineStr"/>
       <c r="O5" s="4" t="inlineStr"/>
@@ -1297,27 +1297,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>DN060</t>
+          <t>DN047</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>DN5060</t>
+          <t>DN5047</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>DN7060</t>
+          <t>DN7047</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>CCAACGTACT</t>
+          <t>TGGCGGACAT</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>ATCATCGACT</t>
+          <t>AGGAAGGTCC</t>
         </is>
       </c>
       <c r="G6" s="4">
@@ -1328,22 +1328,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F6,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>-6.8</v>
+        <v>-5.74</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>-3.89</v>
+        <v>-4.17</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>-2.05</v>
+        <v>-1.62</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>82535</v>
+        <v>45922</v>
       </c>
       <c r="N6" s="4" t="inlineStr"/>
       <c r="O6" s="4" t="inlineStr"/>
@@ -1434,27 +1434,27 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>DN066</t>
+          <t>DN060</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>DN5066</t>
+          <t>DN5060</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>DN7066</t>
+          <t>DN7060</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>TAGTAGGAAC</t>
+          <t>CCAACGTACT</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>GCGGTGAGTT</t>
+          <t>ATCATCGACT</t>
         </is>
       </c>
       <c r="G7" s="4">
@@ -1467,20 +1467,20 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-5.95</v>
+        <v>-6.8</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>-4.95</v>
+        <v>-3.89</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>-1.59</v>
+        <v>-2.05</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>89516</v>
+        <v>82535</v>
       </c>
       <c r="N7" s="4" t="inlineStr"/>
       <c r="O7" s="4" t="inlineStr"/>
@@ -1571,27 +1571,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>DN072</t>
+          <t>DN063</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>DN5072</t>
+          <t>DN5063</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>DN7072</t>
+          <t>DN7063</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>TACACTATCC</t>
+          <t>TTGGTCAGGA</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>ATATACGTGC</t>
+          <t>ACGTTAGACA</t>
         </is>
       </c>
       <c r="G8" s="4">
@@ -1602,22 +1602,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F8,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>-5.84</v>
+        <v>-6.44</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>-4.54</v>
+        <v>-5.36</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>-2.75</v>
+        <v>-2.61</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>100074</v>
+        <v>46291</v>
       </c>
       <c r="N8" s="4" t="inlineStr"/>
       <c r="O8" s="4" t="inlineStr"/>
@@ -1708,27 +1708,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>DN085</t>
+          <t>DN066</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>DN5085</t>
+          <t>DN5066</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>DN7085</t>
+          <t>DN7066</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>GTGCTGAAGG</t>
+          <t>TAGTAGGAAC</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>TCGACGTAGG</t>
+          <t>GCGGTGAGTT</t>
         </is>
       </c>
       <c r="G9" s="4">
@@ -1739,22 +1739,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F9,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>-7.72</v>
+        <v>-5.95</v>
       </c>
       <c r="K9" s="4" t="n">
-        <v>-3.99</v>
+        <v>-4.95</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>-2.35</v>
+        <v>-1.59</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>99155</v>
+        <v>89516</v>
       </c>
       <c r="N9" s="4" t="inlineStr"/>
       <c r="O9" s="4" t="inlineStr"/>
@@ -1845,27 +1845,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>DN088</t>
+          <t>DN072</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>DN5088</t>
+          <t>DN5072</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>DN7088</t>
+          <t>DN7072</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>ACTGGAGCGA</t>
+          <t>TACACTATCC</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>GTGAGAAGTT</t>
+          <t>ATATACGTGC</t>
         </is>
       </c>
       <c r="G10" s="4">
@@ -1878,20 +1878,20 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>-5.97</v>
+        <v>-5.84</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>-3.83</v>
+        <v>-4.54</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>-1.59</v>
+        <v>-2.75</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>146493</v>
+        <v>100074</v>
       </c>
       <c r="N10" s="4" t="inlineStr"/>
       <c r="O10" s="4" t="inlineStr"/>
@@ -1982,27 +1982,27 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>DN098</t>
+          <t>DN077</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>DN5098</t>
+          <t>DN5077</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>DN7098</t>
+          <t>DN7077</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>AGGTTGGTTA</t>
+          <t>AGGTCACATA</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>CACTCTGACC</t>
+          <t>CGCTGACGAT</t>
         </is>
       </c>
       <c r="G11" s="4">
@@ -2013,22 +2013,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F11,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I11" s="7" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>-6.03</v>
+        <v>-6.26</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>-3.83</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>-1.62</v>
+        <v>-1.59</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>45643</v>
+        <v>55129</v>
       </c>
       <c r="N11" s="4" t="inlineStr"/>
       <c r="O11" s="4" t="inlineStr"/>
@@ -2119,27 +2119,27 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>DN102</t>
+          <t>DN081</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>DN5102</t>
+          <t>DN5081</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>DN7102</t>
+          <t>DN7081</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>CTATCCTCGG</t>
+          <t>CGGAGACGTA</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>GTGCCGCATA</t>
+          <t>GCGGTCTATC</t>
         </is>
       </c>
       <c r="G12" s="4">
@@ -2152,20 +2152,20 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>-8.49</v>
+        <v>-5.74</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>-3.92</v>
+        <v>-3.83</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>-2.61</v>
+        <v>-1.62</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>116812</v>
+        <v>50452</v>
       </c>
       <c r="N12" s="4" t="inlineStr"/>
       <c r="O12" s="4" t="inlineStr"/>
@@ -2256,27 +2256,27 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>DN119</t>
+          <t>DN085</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>DN5119</t>
+          <t>DN5085</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>DN7119</t>
+          <t>DN7085</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>TCAGAATCAC</t>
+          <t>GTGCTGAAGG</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>TGCAAGGAGC</t>
+          <t>TCGACGTAGG</t>
         </is>
       </c>
       <c r="G13" s="4">
@@ -2287,22 +2287,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F13,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>-6.12</v>
+        <v>-7.72</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>-4.95</v>
+        <v>-3.99</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>-1.62</v>
+        <v>-2.35</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>88718</v>
+        <v>99155</v>
       </c>
       <c r="N13" s="4" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
@@ -2393,27 +2393,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>DN121</t>
+          <t>DN088</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>DN5121</t>
+          <t>DN5088</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>DN7121</t>
+          <t>DN7088</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>GTAGTGAGAC</t>
+          <t>ACTGGAGCGA</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>ATTCGGATTG</t>
+          <t>GTGAGAAGTT</t>
         </is>
       </c>
       <c r="G14" s="4">
@@ -2426,20 +2426,20 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>-7.14</v>
+        <v>-5.97</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>-4.95</v>
+        <v>-3.83</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>-1.77</v>
+        <v>-1.59</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>37195</v>
+        <v>146493</v>
       </c>
       <c r="N14" s="4" t="inlineStr"/>
       <c r="O14" s="4" t="inlineStr"/>
@@ -2530,27 +2530,27 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>DN126</t>
+          <t>DN109</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>DN5126</t>
+          <t>DN5109</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>DN7126</t>
+          <t>DN7109</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>GTTACAGGAT</t>
+          <t>TTCCAGTGTT</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>CATTGACGCC</t>
+          <t>GCGCTACTCT</t>
         </is>
       </c>
       <c r="G15" s="4">
@@ -2561,22 +2561,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F15,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>-5.8</v>
+        <v>-6.55</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>-4.17</v>
+        <v>-3.79</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>-1.62</v>
+        <v>-1.59</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>67548</v>
+        <v>59187</v>
       </c>
       <c r="N15" s="4" t="inlineStr"/>
       <c r="O15" s="4" t="inlineStr"/>
@@ -2667,27 +2667,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>DN133</t>
+          <t>DN116</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>DN5133</t>
+          <t>DN5116</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>DN7133</t>
+          <t>DN7116</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>GTCCTAGACC</t>
+          <t>AGTAGCCACC</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>CGTCCTATTG</t>
+          <t>TGCGAATCGG</t>
         </is>
       </c>
       <c r="G16" s="4">
@@ -2698,22 +2698,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F16,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>-6.16</v>
+        <v>-6.52</v>
       </c>
       <c r="K16" s="4" t="n">
         <v>-4.54</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>-1.77</v>
+        <v>-3.69</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>36837</v>
+        <v>45417</v>
       </c>
       <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
@@ -2804,27 +2804,27 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>DN140</t>
+          <t>DN129</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>DN5140</t>
+          <t>DN5129</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>DN7140</t>
+          <t>DN7129</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>ATACCTCTGT</t>
+          <t>AGGTGAGGAG</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>TTATCTTGCG</t>
+          <t>AGGACCAGAA</t>
         </is>
       </c>
       <c r="G17" s="4">
@@ -2837,20 +2837,20 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>-6.34</v>
+        <v>-8.27</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>-3.96</v>
+        <v>-4.02</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>-1.77</v>
+        <v>-2.61</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>55590</v>
+        <v>130743</v>
       </c>
       <c r="N17" s="4" t="inlineStr"/>
       <c r="O17" s="4" t="inlineStr"/>
@@ -2941,27 +2941,27 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>DN144</t>
+          <t>DN135</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>DN5144</t>
+          <t>DN5135</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>DN7144</t>
+          <t>DN7135</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>TACGGTGAGG</t>
+          <t>AGGCCTCAAG</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>GTCACCTGTA</t>
+          <t>AAGGTACAAC</t>
         </is>
       </c>
       <c r="G18" s="4">
@@ -2974,20 +2974,20 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>-7.87</v>
+        <v>-6.72</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>-4.99</v>
+        <v>-4.02</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>-2.61</v>
+        <v>-1.62</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>111405</v>
+        <v>121927</v>
       </c>
       <c r="N18" s="4" t="inlineStr"/>
       <c r="O18" s="4" t="inlineStr"/>
@@ -3078,27 +3078,27 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>DN165</t>
+          <t>DN140</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>DN5165</t>
+          <t>DN5140</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>DN7165</t>
+          <t>DN7140</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>GCTTAGGTAA</t>
+          <t>ATACCTCTGT</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>AGAGCAACTA</t>
+          <t>TTATCTTGCG</t>
         </is>
       </c>
       <c r="G19" s="4">
@@ -3109,22 +3109,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F19,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I19" s="7" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>-6.67</v>
+        <v>-6.34</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>-4</v>
+        <v>-3.96</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>-2.61</v>
+        <v>-1.77</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>132144</v>
+        <v>55590</v>
       </c>
       <c r="N19" s="4" t="inlineStr"/>
       <c r="O19" s="4" t="inlineStr"/>
@@ -3215,27 +3215,27 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>DN169</t>
+          <t>DN165</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>DN5169</t>
+          <t>DN5165</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>DN7169</t>
+          <t>DN7165</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>TGGCCACCTT</t>
+          <t>GCTTAGGTAA</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>CGATTACTAG</t>
+          <t>AGAGCAACTA</t>
         </is>
       </c>
       <c r="G20" s="4">
@@ -3246,22 +3246,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F20,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>-5.93</v>
+        <v>-6.67</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>-3.99</v>
+        <v>-4</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>-1.77</v>
+        <v>-2.61</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>36304</v>
+        <v>132144</v>
       </c>
       <c r="N20" s="4" t="inlineStr"/>
       <c r="O20" s="4" t="inlineStr"/>
@@ -3352,27 +3352,27 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>DN174</t>
+          <t>DN180</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>DN5174</t>
+          <t>DN5180</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>DN7174</t>
+          <t>DN7180</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>TGCCATATCT</t>
+          <t>CGCGAGTATG</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>CAGGATCGCT</t>
+          <t>CACCTACTTA</t>
         </is>
       </c>
       <c r="G21" s="4">
@@ -3385,20 +3385,20 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>-5.95</v>
+        <v>-7.97</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>-3.78</v>
+        <v>-5.22</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>-2.51</v>
+        <v>-2.61</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>146815</v>
+        <v>121767</v>
       </c>
       <c r="N21" s="4" t="inlineStr"/>
       <c r="O21" s="4" t="inlineStr"/>
@@ -3489,27 +3489,27 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>DN181</t>
+          <t>DN184</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>DN5181</t>
+          <t>DN5184</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>DN7181</t>
+          <t>DN7184</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>CACCACGGTT</t>
+          <t>CAACGATTGA</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>CAGCTAGAAT</t>
+          <t>AATCTCCGAA</t>
         </is>
       </c>
       <c r="G22" s="4">
@@ -3520,22 +3520,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F22,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>-6.54</v>
+        <v>-6.68</v>
       </c>
       <c r="K22" s="4" t="n">
-        <v>-3.79</v>
+        <v>-3.83</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>-1.59</v>
+        <v>-2.61</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>63975</v>
+        <v>45309</v>
       </c>
       <c r="N22" s="4" t="inlineStr"/>
       <c r="O22" s="4" t="inlineStr"/>
@@ -3626,27 +3626,27 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>DN192</t>
+          <t>DN190</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>DN5192</t>
+          <t>DN5190</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>DN7192</t>
+          <t>DN7190</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>CTCAGCCAGT</t>
+          <t>GCAAGCCAAC</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>CAACCTGCAC</t>
+          <t>TGCTAGCCAT</t>
         </is>
       </c>
       <c r="G23" s="4">
@@ -3659,20 +3659,20 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>-6.89</v>
+        <v>-7.64</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>-3.8</v>
+        <v>-4.95</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>-1.62</v>
+        <v>-1.59</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>45763</v>
+        <v>105502</v>
       </c>
       <c r="N23" s="4" t="inlineStr"/>
       <c r="O23" s="4" t="inlineStr"/>
@@ -3763,27 +3763,27 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>DN197</t>
+          <t>DN199</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>DN5197</t>
+          <t>DN5199</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>DN7197</t>
+          <t>DN7199</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>GTTGAACGTA</t>
+          <t>GTAAGATGAG</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>CAAGACTCTA</t>
+          <t>TCACTGCTAG</t>
         </is>
       </c>
       <c r="G24" s="4">
@@ -3796,20 +3796,20 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>-5.92</v>
+        <v>-8.09</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>-3.83</v>
+        <v>-4.19</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>-2.61</v>
+        <v>-1.77</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>81594</v>
+        <v>348523</v>
       </c>
       <c r="N24" s="4" t="inlineStr"/>
       <c r="O24" s="4" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F25,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -4037,27 +4037,27 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>DN209</t>
+          <t>DN232</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>DN5209</t>
+          <t>DN5232</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>DN7209</t>
+          <t>DN7232</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>GTGTTAACTG</t>
+          <t>GCACCGTCAA</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>ATGGTCCACG</t>
+          <t>GCCAAGTCCA</t>
         </is>
       </c>
       <c r="G26" s="4">
@@ -4070,20 +4070,20 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>-8.09</v>
+        <v>-6.44</v>
       </c>
       <c r="K26" s="4" t="n">
-        <v>-4.92</v>
+        <v>-3.83</v>
       </c>
       <c r="L26" s="4" t="n">
-        <v>-1.69</v>
+        <v>-2.61</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>141823</v>
+        <v>108488</v>
       </c>
       <c r="N26" s="4" t="inlineStr"/>
       <c r="O26" s="4" t="inlineStr"/>
@@ -4174,27 +4174,27 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>DN232</t>
+          <t>DN245</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>DN5232</t>
+          <t>DN5245</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>DN7232</t>
+          <t>DN7245</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>GCACCGTCAA</t>
+          <t>CTTGCCAACT</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>GCCAAGTCCA</t>
+          <t>GTGCGTTACC</t>
         </is>
       </c>
       <c r="G27" s="4">
@@ -4205,22 +4205,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F27,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>-6.44</v>
+        <v>-6.27</v>
       </c>
       <c r="K27" s="4" t="n">
         <v>-3.83</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>-2.61</v>
+        <v>-2.05</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>108488</v>
+        <v>96963</v>
       </c>
       <c r="N27" s="4" t="inlineStr"/>
       <c r="O27" s="4" t="inlineStr"/>
@@ -4311,27 +4311,27 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>DN239</t>
+          <t>DN259</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>DN5239</t>
+          <t>DN5259</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>DN7239</t>
+          <t>DN7259</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>ACTCATGGAA</t>
+          <t>GTCCACAGAA</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>CGGTAGTCAG</t>
+          <t>GAGCCAAGTC</t>
         </is>
       </c>
       <c r="G28" s="4">
@@ -4342,22 +4342,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F28,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>-6.27</v>
+        <v>-6.15</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>-3.99</v>
+        <v>-4.43</v>
       </c>
       <c r="L28" s="4" t="n">
-        <v>-1.77</v>
+        <v>-2.05</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>57075</v>
+        <v>60711</v>
       </c>
       <c r="N28" s="4" t="inlineStr"/>
       <c r="O28" s="4" t="inlineStr"/>
@@ -4448,27 +4448,27 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>DN245</t>
+          <t>DN266</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>DN5245</t>
+          <t>DN5266</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>DN7245</t>
+          <t>DN7266</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>CTTGCCAACT</t>
+          <t>GCAACTTATC</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>GTGCGTTACC</t>
+          <t>ACCAGTTCCG</t>
         </is>
       </c>
       <c r="G29" s="4">
@@ -4481,20 +4481,20 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>-6.27</v>
+        <v>-7.87</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>-3.83</v>
+        <v>-4.7</v>
       </c>
       <c r="L29" s="4" t="n">
-        <v>-2.05</v>
+        <v>-1.77</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>96963</v>
+        <v>39480</v>
       </c>
       <c r="N29" s="4" t="inlineStr"/>
       <c r="O29" s="4" t="inlineStr"/>
@@ -4585,27 +4585,27 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>DN257</t>
+          <t>DN273</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>DN5257</t>
+          <t>DN5273</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>DN7257</t>
+          <t>DN7273</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>TCTCTAATGC</t>
+          <t>AGAGCTGTCC</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>TGCTCAGAAC</t>
+          <t>GACGAGTGAA</t>
         </is>
       </c>
       <c r="G30" s="4">
@@ -4616,22 +4616,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F30,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J30" s="4" t="n">
-        <v>-6.45</v>
+        <v>-6.53</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>-4.78</v>
+        <v>-4.54</v>
       </c>
       <c r="L30" s="4" t="n">
-        <v>-1.62</v>
+        <v>-2.61</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>71251</v>
+        <v>71759</v>
       </c>
       <c r="N30" s="4" t="inlineStr"/>
       <c r="O30" s="4" t="inlineStr"/>
@@ -4722,27 +4722,27 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>DN259</t>
+          <t>DN319</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>DN5259</t>
+          <t>DN5319</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>DN7259</t>
+          <t>DN7319</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>GTCCACAGAA</t>
+          <t>GTGCACCACT</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>GAGCCAAGTC</t>
+          <t>CGTTCATGCG</t>
         </is>
       </c>
       <c r="G31" s="4">
@@ -4753,22 +4753,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F31,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I31" s="7" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>-6.15</v>
+        <v>-6.34</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>-4.43</v>
+        <v>-4.21</v>
       </c>
       <c r="L31" s="4" t="n">
         <v>-2.05</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>60711</v>
+        <v>52945</v>
       </c>
       <c r="N31" s="4" t="inlineStr"/>
       <c r="O31" s="4" t="inlineStr"/>
@@ -4859,27 +4859,27 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>DN267</t>
+          <t>DN326</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>DN5267</t>
+          <t>DN5326</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>DN7267</t>
+          <t>DN7326</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>GAAGCAATTG</t>
+          <t>CGACTGCCTA</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>ACTATTGAGG</t>
+          <t>GTCGGTAATA</t>
         </is>
       </c>
       <c r="G32" s="4">
@@ -4892,20 +4892,20 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>-8.119999999999999</v>
+        <v>-6.44</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>-4.74</v>
+        <v>-3.83</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>-2.35</v>
+        <v>-2.61</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>146009</v>
+        <v>75074</v>
       </c>
       <c r="N32" s="4" t="inlineStr"/>
       <c r="O32" s="4" t="inlineStr"/>
@@ -4996,27 +4996,27 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>DN277</t>
+          <t>DN349</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>DN5277</t>
+          <t>DN5349</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>DN7277</t>
+          <t>DN7349</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>CTCATATGTC</t>
+          <t>TGAAGCCTAA</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>AGACGATAGC</t>
+          <t>TGAGCGATTC</t>
         </is>
       </c>
       <c r="G33" s="4">
@@ -5029,20 +5029,20 @@
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>-7.81</v>
+        <v>-6.59</v>
       </c>
       <c r="K33" s="4" t="n">
-        <v>-4.7</v>
+        <v>-3.83</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>-1.62</v>
+        <v>-2.19</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>84107</v>
+        <v>69590</v>
       </c>
       <c r="N33" s="4" t="inlineStr"/>
       <c r="O33" s="4" t="inlineStr"/>
@@ -5133,27 +5133,27 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>DN280</t>
+          <t>DN364</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>DN5280</t>
+          <t>DN5364</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>DN7280</t>
+          <t>DN7364</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>AATCCTTCCT</t>
+          <t>AACCTCATTG</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>GTAACTCCAA</t>
+          <t>ATGCAGGACG</t>
         </is>
       </c>
       <c r="G34" s="4">
@@ -5166,20 +5166,20 @@
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>-6.93</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>-3.78</v>
+        <v>-4.13</v>
       </c>
       <c r="L34" s="4" t="n">
-        <v>-2.61</v>
+        <v>-1.69</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>81002</v>
+        <v>144051</v>
       </c>
       <c r="N34" s="4" t="inlineStr"/>
       <c r="O34" s="4" t="inlineStr"/>
@@ -5270,27 +5270,27 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>DN294</t>
+          <t>DN365</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>DN5294</t>
+          <t>DN5365</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>DN7294</t>
+          <t>DN7365</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>GCATCGAAGG</t>
+          <t>CGTGGTTGGA</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>TTCTCCAAGA</t>
+          <t>CTAGATGCGG</t>
         </is>
       </c>
       <c r="G35" s="4">
@@ -5303,20 +5303,20 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>-7.81</v>
+        <v>-6.54</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>-4.57</v>
+        <v>-4.43</v>
       </c>
       <c r="L35" s="4" t="n">
-        <v>-2.61</v>
+        <v>-3.3</v>
       </c>
       <c r="M35" s="4" t="n">
-        <v>112640</v>
+        <v>41183</v>
       </c>
       <c r="N35" s="4" t="inlineStr"/>
       <c r="O35" s="4" t="inlineStr"/>
@@ -5407,27 +5407,27 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>DN302</t>
+          <t>DN371</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>DN5302</t>
+          <t>DN5371</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>DN7302</t>
+          <t>DN7371</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>GACGGTTACT</t>
+          <t>GCAATGCGCT</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>GCGGACTCAA</t>
+          <t>ATCAGGTCAA</t>
         </is>
       </c>
       <c r="G36" s="4">
@@ -5438,7 +5438,7 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F36,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I36" s="7" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -5447,13 +5447,13 @@
         <v>-7</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>-3.78</v>
+        <v>-4.43</v>
       </c>
       <c r="L36" s="4" t="n">
         <v>-2.61</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>60603</v>
+        <v>61623</v>
       </c>
       <c r="N36" s="4" t="inlineStr"/>
       <c r="O36" s="4" t="inlineStr"/>
@@ -5544,27 +5544,27 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>DN311</t>
+          <t>DN378</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>DN5311</t>
+          <t>DN5378</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>DN7311</t>
+          <t>DN7378</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>TGACCTTCTA</t>
+          <t>GTCGTTGTGG</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>GTTCATCATC</t>
+          <t>GATGCTCAGT</t>
         </is>
       </c>
       <c r="G37" s="4">
@@ -5577,20 +5577,20 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>-6.03</v>
+        <v>-7.64</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>-3.83</v>
+        <v>-4.66</v>
       </c>
       <c r="L37" s="4" t="n">
-        <v>-1.62</v>
+        <v>-1.59</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>59229</v>
+        <v>125089</v>
       </c>
       <c r="N37" s="4" t="inlineStr"/>
       <c r="O37" s="4" t="inlineStr"/>
@@ -5681,27 +5681,27 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>DN325</t>
+          <t>DN381</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>DN5325</t>
+          <t>DN5381</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>DN7325</t>
+          <t>DN7381</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>GCGATACAGG</t>
+          <t>AGAGAAGGAA</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>GCGATTAGCC</t>
+          <t>GCGCATAGTG</t>
         </is>
       </c>
       <c r="G38" s="4">
@@ -5714,20 +5714,20 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>-7.28</v>
+        <v>-6.27</v>
       </c>
       <c r="K38" s="4" t="n">
-        <v>-3.99</v>
+        <v>-3.93</v>
       </c>
       <c r="L38" s="4" t="n">
-        <v>-1.62</v>
+        <v>-1.77</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>127676</v>
+        <v>36559</v>
       </c>
       <c r="N38" s="4" t="inlineStr"/>
       <c r="O38" s="4" t="inlineStr"/>
@@ -5818,27 +5818,27 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>DN326</t>
+          <t>DN392</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>DN5326</t>
+          <t>DN5392</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>DN7326</t>
+          <t>DN7392</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>CGACTGCCTA</t>
+          <t>CGCGATGAGA</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>GTCGGTAATA</t>
+          <t>CCAGGAGAAC</t>
         </is>
       </c>
       <c r="G39" s="4">
@@ -5849,22 +5849,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F39,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>-6.44</v>
+        <v>-6.11</v>
       </c>
       <c r="K39" s="4" t="n">
         <v>-3.83</v>
       </c>
       <c r="L39" s="4" t="n">
-        <v>-2.61</v>
+        <v>-1.62</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>75074</v>
+        <v>49126</v>
       </c>
       <c r="N39" s="4" t="inlineStr"/>
       <c r="O39" s="4" t="inlineStr"/>
@@ -5955,27 +5955,27 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>DN349</t>
+          <t>DN409</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>DN5349</t>
+          <t>DN5409</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>DN7349</t>
+          <t>DN7409</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>TGAAGCCTAA</t>
+          <t>TCGAACACTT</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>TGAGCGATTC</t>
+          <t>TGCACAAGCG</t>
         </is>
       </c>
       <c r="G40" s="4">
@@ -5986,22 +5986,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F40,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I40" s="7" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>-6.59</v>
+        <v>-6.39</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>-3.83</v>
+        <v>-4.18</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>-2.19</v>
+        <v>-1.77</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>69590</v>
+        <v>52409</v>
       </c>
       <c r="N40" s="4" t="inlineStr"/>
       <c r="O40" s="4" t="inlineStr"/>
@@ -6092,27 +6092,27 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>DN359</t>
+          <t>DN414</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>DN5359</t>
+          <t>DN5414</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>DN7359</t>
+          <t>DN7414</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>GCGCTTGTTC</t>
+          <t>GAACTTACAG</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>ACCGGTCGAT</t>
+          <t>ACGAATCCAT</t>
         </is>
       </c>
       <c r="G41" s="4">
@@ -6123,22 +6123,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F41,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I41" s="6" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>-6.11</v>
+        <v>-8.15</v>
       </c>
       <c r="K41" s="4" t="n">
-        <v>-5</v>
+        <v>-4.31</v>
       </c>
       <c r="L41" s="4" t="n">
         <v>-1.59</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>63627</v>
+        <v>133197</v>
       </c>
       <c r="N41" s="4" t="inlineStr"/>
       <c r="O41" s="4" t="inlineStr"/>
@@ -6229,27 +6229,27 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>DN365</t>
+          <t>DN422</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>DN5365</t>
+          <t>DN5422</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>DN7365</t>
+          <t>DN7422</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>CGTGGTTGGA</t>
+          <t>ACACGGAGGT</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>CTAGATGCGG</t>
+          <t>TCTTGATTGG</t>
         </is>
       </c>
       <c r="G42" s="4">
@@ -6260,22 +6260,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F42,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I42" s="7" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J42" s="4" t="n">
-        <v>-6.54</v>
+        <v>-6.38</v>
       </c>
       <c r="K42" s="4" t="n">
-        <v>-4.43</v>
+        <v>-3.89</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>-3.3</v>
+        <v>-2.3</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>41183</v>
+        <v>42109</v>
       </c>
       <c r="N42" s="4" t="inlineStr"/>
       <c r="O42" s="4" t="inlineStr"/>
@@ -6366,27 +6366,27 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>DN366</t>
+          <t>DN438</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>DN5366</t>
+          <t>DN5438</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>DN7366</t>
+          <t>DN7438</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>TGGTGCCTTC</t>
+          <t>ATGACTATGG</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>CGCAGTCCAA</t>
+          <t>CCTCGAAGTG</t>
         </is>
       </c>
       <c r="G43" s="4">
@@ -6397,22 +6397,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F43,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I43" s="6" t="inlineStr">
+      <c r="I43" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>-6.93</v>
+        <v>-7.72</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>-4.7</v>
+        <v>-3.93</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>-2.61</v>
+        <v>-1.77</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>60491</v>
+        <v>109448</v>
       </c>
       <c r="N43" s="4" t="inlineStr"/>
       <c r="O43" s="4" t="inlineStr"/>
@@ -6503,27 +6503,27 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>DN392</t>
+          <t>DN450</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>DN5392</t>
+          <t>DN5450</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>DN7392</t>
+          <t>DN7450</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>CGCGATGAGA</t>
+          <t>GATTCGGATT</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>CCAGGAGAAC</t>
+          <t>AGGATTACTC</t>
         </is>
       </c>
       <c r="G44" s="4">
@@ -6534,22 +6534,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F44,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I44" s="7" t="inlineStr">
+      <c r="I44" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>-6.11</v>
+        <v>-6.22</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>-3.83</v>
+        <v>-3.79</v>
       </c>
       <c r="L44" s="4" t="n">
         <v>-1.62</v>
       </c>
       <c r="M44" s="4" t="n">
-        <v>49126</v>
+        <v>59960</v>
       </c>
       <c r="N44" s="4" t="inlineStr"/>
       <c r="O44" s="4" t="inlineStr"/>
@@ -6640,27 +6640,27 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>DN422</t>
+          <t>DN452</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>DN5422</t>
+          <t>DN5452</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>DN7422</t>
+          <t>DN7452</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>ACACGGAGGT</t>
+          <t>AAGTCGGAGG</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>TCTTGATTGG</t>
+          <t>TATCTAGAGG</t>
         </is>
       </c>
       <c r="G45" s="4">
@@ -6673,20 +6673,20 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>-6.38</v>
+        <v>-7.34</v>
       </c>
       <c r="K45" s="4" t="n">
-        <v>-3.89</v>
+        <v>-4.16</v>
       </c>
       <c r="L45" s="4" t="n">
-        <v>-2.3</v>
+        <v>-2.35</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>42109</v>
+        <v>85153</v>
       </c>
       <c r="N45" s="4" t="inlineStr"/>
       <c r="O45" s="4" t="inlineStr"/>
@@ -6777,27 +6777,27 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>DN443</t>
+          <t>DN454</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>DN5443</t>
+          <t>DN5454</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>DN7443</t>
+          <t>DN7454</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>AATACCAAGG</t>
+          <t>CACCTTGTCC</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>AATTCCGGTT</t>
+          <t>ACATTCTAGC</t>
         </is>
       </c>
       <c r="G46" s="4">
@@ -6808,22 +6808,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F46,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I46" s="6" t="inlineStr">
+      <c r="I46" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>-7.96</v>
+        <v>-6.03</v>
       </c>
       <c r="K46" s="4" t="n">
-        <v>-5</v>
+        <v>-4.54</v>
       </c>
       <c r="L46" s="4" t="n">
-        <v>-1.59</v>
+        <v>-1.62</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>102474</v>
+        <v>81693</v>
       </c>
       <c r="N46" s="4" t="inlineStr"/>
       <c r="O46" s="4" t="inlineStr"/>
@@ -6914,27 +6914,27 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>DN452</t>
+          <t>DN471</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>DN5452</t>
+          <t>DN5471</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>DN7452</t>
+          <t>DN7471</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>AAGTCGGAGG</t>
+          <t>GAACGCAACC</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>TATCTAGAGG</t>
+          <t>TCGTCCATCC</t>
         </is>
       </c>
       <c r="G47" s="4">
@@ -6945,22 +6945,22 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F47,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I47" s="6" t="inlineStr">
+      <c r="I47" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>-7.34</v>
+        <v>-5.74</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>-4.16</v>
+        <v>-4.54</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>-2.35</v>
+        <v>-1.62</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>85153</v>
+        <v>47469</v>
       </c>
       <c r="N47" s="4" t="inlineStr"/>
       <c r="O47" s="4" t="inlineStr"/>
@@ -7051,27 +7051,27 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>DN456</t>
+          <t>DN472</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>DN5456</t>
+          <t>DN5472</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>DN7456</t>
+          <t>DN7472</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>ACCGAACACC</t>
+          <t>TGTGATAGGT</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>GCAGCACGAA</t>
+          <t>TTGTCGTGTA</t>
         </is>
       </c>
       <c r="G48" s="4">
@@ -7084,20 +7084,20 @@
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>-6.43</v>
+        <v>-6.36</v>
       </c>
       <c r="K48" s="4" t="n">
-        <v>-4.54</v>
+        <v>-4.32</v>
       </c>
       <c r="L48" s="4" t="n">
         <v>-2.61</v>
       </c>
       <c r="M48" s="4" t="n">
-        <v>45609</v>
+        <v>69196</v>
       </c>
       <c r="N48" s="4" t="inlineStr"/>
       <c r="O48" s="4" t="inlineStr"/>
@@ -7188,27 +7188,27 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>DN478</t>
+          <t>DN477</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>DN5478</t>
+          <t>DN5477</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>DN7478</t>
+          <t>DN7477</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>CTCCGAGTAA</t>
+          <t>AGTCAGCCTT</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>AGTAGAATCC</t>
+          <t>CTTACTGGAC</t>
         </is>
       </c>
       <c r="G49" s="4">
@@ -7219,7 +7219,7 @@
         <f>LEN(SUBSTITUTE(SUBSTITUTE(F49,"A",""),"T",""))</f>
         <v/>
       </c>
-      <c r="I49" s="7" t="inlineStr">
+      <c r="I49" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -7228,13 +7228,13 @@
         <v>-5.74</v>
       </c>
       <c r="K49" s="4" t="n">
-        <v>-3.83</v>
+        <v>-3.79</v>
       </c>
       <c r="L49" s="4" t="n">
         <v>-1.62</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>46270</v>
+        <v>58722</v>
       </c>
       <c r="N49" s="4" t="inlineStr"/>
       <c r="O49" s="4" t="inlineStr"/>

</xml_diff>